<commit_message>
Label hypothetical figures, fill RICE ranks, add charts and README
- Workbook labelled as a course project; stakeholder counts and targets marked hypothetical
- Filled the empty Rank column; stated the goal as +15 percentage points (62% to 77%)
- Added 4 charts, the chart script, requirements.txt and a full README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WF4k7piiwojb9edAdFVsTN
</commit_message>
<xml_diff>
--- a/03_Feature_Prioritization_Roadmap.xlsx
+++ b/03_Feature_Prioritization_Roadmap.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="164">
-  <si>
-    <t xml:space="preserve">EdTech Platform — Feature Backlog (MBA Capstone)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stakeholder sources: Students (n=120), Instructors (n=18), Administrators (n=6)  |  Scoring: RICE + MoSCoW  |  Target: +15% course completion rate</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="166">
+  <si>
+    <t xml:space="preserve">EdTech Platform — Feature Backlog (Course Project)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypothetical stakeholder sources: Students (n=120), Instructors (n=18), Administrators (n=6)  |  Scoring: RICE + MoSCoW  |  Target: +15 percentage points course completion (62% to 77%)</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -376,7 +376,10 @@
     <t xml:space="preserve">Live Streaming</t>
   </si>
   <si>
-    <t xml:space="preserve">Success Metrics &amp; Acceptance Criteria — Target: +15% Course Completion Rate</t>
+    <t xml:space="preserve">Rank compares the 12 features on this sheet. Feature_Backlog scores all 25 items; the roadmap takes all 8 Must Haves plus 4 Should Haves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Success Metrics &amp; Acceptance Criteria — Target: +15 Percentage Points Course Completion (62% to 77%)</t>
   </si>
   <si>
     <t xml:space="preserve">Primary KPI</t>
@@ -515,18 +518,22 @@
   </si>
   <si>
     <t xml:space="preserve">Aggregate lift across all 12 initiatives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All baselines and targets are hypothetical planning figures for an illustrative platform.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
+    <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -666,6 +673,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
@@ -746,11 +761,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -763,51 +782,51 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -823,19 +842,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -851,19 +870,31 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1122,980 +1153,980 @@
   <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="6" t="n">
         <f aca="false">(E5*F5*(G5/100))/H5</f>
         <v>320</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>950</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>90</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="9" t="n">
         <f aca="false">(E6*F6*(G6/100))/H6</f>
         <v>641.25</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>1100</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I7" s="6" t="n">
         <f aca="false">(E7*F7*(G7/100))/H7</f>
         <v>192.5</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="9" t="n">
         <f aca="false">(E8*F8*(G8/100))/H8</f>
         <v>855</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="J8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>180</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="6" t="n">
         <f aca="false">(E9*F9*(G9/100))/H9</f>
         <v>91.8</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="8" t="n">
         <v>750</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="9" t="n">
         <f aca="false">(E10*F10*(G10/100))/H10</f>
         <v>121.875</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <v>75</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="H11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="6" t="n">
         <f aca="false">(E11*F11*(G11/100))/H11</f>
         <v>150</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="9" t="n">
         <f aca="false">(E12*F12*(G12/100))/H12</f>
         <v>60</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="I13" s="6" t="n">
         <f aca="false">(E13*F13*(G13/100))/H13</f>
         <v>82.5</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="8" t="n">
         <v>90</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="9" t="n">
         <f aca="false">(E14*F14*(G14/100))/H14</f>
         <v>54</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="H15" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="6" t="n">
         <f aca="false">(E15*F15*(G15/100))/H15</f>
         <v>42</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="8" t="n">
         <v>1100</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G16" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="9" t="n">
         <f aca="false">(E16*F16*(G16/100))/H16</f>
         <v>391.875</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="J16" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="H17" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I17" s="6" t="n">
         <f aca="false">(E17*F17*(G17/100))/H17</f>
         <v>30</v>
       </c>
-      <c r="J17" s="12" t="s">
+      <c r="J17" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E18" s="8" t="n">
         <v>450</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F18" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H18" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="9" t="n">
         <f aca="false">(E18*F18*(G18/100))/H18</f>
         <v>83.5714285714286</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>900</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="H19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I19" s="6" t="n">
         <f aca="false">(E19*F19*(G19/100))/H19</f>
         <v>765</v>
       </c>
-      <c r="J19" s="6" t="s">
+      <c r="J19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="E20" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G20" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H20" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="9" t="n">
         <f aca="false">(E20*F20*(G20/100))/H20</f>
         <v>320</v>
       </c>
-      <c r="J20" s="13" t="s">
+      <c r="J20" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="K20" s="7" t="s">
+      <c r="K20" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="H21" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="6" t="n">
         <f aca="false">(E21*F21*(G21/100))/H21</f>
         <v>18.75</v>
       </c>
-      <c r="J21" s="12" t="s">
+      <c r="J21" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="K21" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="E22" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F22" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G22" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H22" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="9" t="n">
         <f aca="false">(E22*F22*(G22/100))/H22</f>
         <v>96</v>
       </c>
-      <c r="J22" s="10" t="s">
+      <c r="J22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="G23" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="H23" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="I23" s="6" t="n">
         <f aca="false">(E23*F23*(G23/100))/H23</f>
         <v>6.42857142857143</v>
       </c>
-      <c r="J23" s="14" t="s">
+      <c r="J23" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="K23" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="E24" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="F24" s="7" t="n">
+      <c r="F24" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="7" t="n">
+      <c r="G24" s="8" t="n">
         <v>55</v>
       </c>
-      <c r="H24" s="7" t="n">
+      <c r="H24" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="9" t="n">
         <f aca="false">(E24*F24*(G24/100))/H24</f>
         <v>27.5</v>
       </c>
-      <c r="J24" s="15" t="s">
+      <c r="J24" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K24" s="8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="F25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="G25" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="H25" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="I25" s="6" t="n">
         <f aca="false">(E25*F25*(G25/100))/H25</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="J25" s="14" t="s">
+      <c r="J25" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="K25" s="4" t="s">
+      <c r="K25" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="E26" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="F26" s="7" t="n">
+      <c r="F26" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="7" t="n">
+      <c r="G26" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="H26" s="7" t="n">
+      <c r="H26" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I26" s="8" t="n">
+      <c r="I26" s="9" t="n">
         <f aca="false">(E26*F26*(G26/100))/H26</f>
         <v>168</v>
       </c>
-      <c r="J26" s="13" t="s">
+      <c r="J26" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="K26" s="7" t="s">
+      <c r="K26" s="8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="5" t="n">
         <v>180</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="F27" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="G27" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="H27" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="6" t="n">
         <f aca="false">(E27*F27*(G27/100))/H27</f>
         <v>58.5</v>
       </c>
-      <c r="J27" s="12" t="s">
+      <c r="J27" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="K27" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="E28" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="F28" s="7" t="n">
+      <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="7" t="n">
+      <c r="G28" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="H28" s="7" t="n">
+      <c r="H28" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I28" s="8" t="n">
+      <c r="I28" s="9" t="n">
         <f aca="false">(E28*F28*(G28/100))/H28</f>
         <v>360</v>
       </c>
-      <c r="J28" s="13" t="s">
+      <c r="J28" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="K28" s="7" t="s">
+      <c r="K28" s="8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F29" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="G29" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="H29" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="6" t="n">
         <f aca="false">(E29*F29*(G29/100))/H29</f>
         <v>25</v>
       </c>
-      <c r="J29" s="14" t="s">
+      <c r="J29" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="K29" s="4" t="s">
+      <c r="K29" s="5" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2122,356 +2153,356 @@
   <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="5" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="19" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="8" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="8" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2497,350 +2528,403 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="28" t="n">
         <v>0.8</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <f aca="false">(C6*D6*E6)/F6</f>
         <v>320</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="H6" s="29" t="n">
+        <f aca="false">RANK(G6,$G$6:$G$17)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>950</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="30" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="6" t="n">
         <f aca="false">(C7*D7*E7)/F7</f>
         <v>641.25</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="H7" s="31" t="n">
+        <f aca="false">RANK(G7,$G$6:$G$17)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="28" t="n">
         <v>0.85</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <f aca="false">(C8*D8*E8)/F8</f>
         <v>765</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="H8" s="29" t="n">
+        <f aca="false">RANK(G8,$G$6:$G$17)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>900</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="30" t="n">
         <v>0.95</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="6" t="n">
         <f aca="false">(C9*D9*E9)/F9</f>
         <v>855</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="H9" s="31" t="n">
+        <f aca="false">RANK(G9,$G$6:$G$17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="8" t="n">
         <v>1100</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="9" t="n">
         <f aca="false">(C10*D10*E10)/F10</f>
         <v>192.5</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="H10" s="29" t="n">
+        <f aca="false">RANK(G10,$G$6:$G$17)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>180</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="28" t="n">
+      <c r="E11" s="30" t="n">
         <v>0.85</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <f aca="false">(C11*D11*E11)/F11</f>
         <v>91.8</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="H11" s="31" t="n">
+        <f aca="false">RANK(G11,$G$6:$G$17)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <v>750</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="28" t="n">
         <v>0.65</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <f aca="false">(C12*D12*E12)/F12</f>
         <v>121.875</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="H12" s="29" t="n">
+        <f aca="false">RANK(G12,$G$6:$G$17)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>450</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="30" t="n">
         <v>0.65</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <f aca="false">(C13*D13*E13)/F13</f>
         <v>83.5714285714286</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="H13" s="31" t="n">
+        <f aca="false">RANK(G13,$G$6:$G$17)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="9" t="n">
         <f aca="false">(C14*D14*E14)/F14</f>
         <v>150</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="H14" s="29" t="n">
+        <f aca="false">RANK(G14,$G$6:$G$17)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="28" t="n">
+      <c r="E15" s="30" t="n">
         <v>0.7</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <f aca="false">(C15*D15*E15)/F15</f>
         <v>42</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="H15" s="31" t="n">
+        <f aca="false">RANK(G15,$G$6:$G$17)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="9" t="n">
         <f aca="false">(C16*D16*E16)/F16</f>
         <v>168</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="H16" s="29" t="n">
+        <f aca="false">RANK(G16,$G$6:$G$17)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="28" t="n">
+      <c r="E17" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="6" t="n">
         <f aca="false">(C17*D17*E17)/F17</f>
         <v>30</v>
+      </c>
+      <c r="H17" s="31" t="n">
+        <f aca="false">RANK(G17,$G$6:$G$17)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="32" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2863,227 +2947,232 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A1" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>121</v>
       </c>
+      <c r="E3" s="4" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>125</v>
       </c>
+      <c r="E4" s="8" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>129</v>
       </c>
+      <c r="E5" s="5" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>133</v>
       </c>
+      <c r="E6" s="8" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>138</v>
       </c>
+      <c r="E7" s="5" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>162</v>
-      </c>
-      <c r="E14" s="29" t="s">
+      <c r="C14" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="33" t="s">
         <v>163</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>